<commit_message>
update data set and plots
</commit_message>
<xml_diff>
--- a/data/papers_summary.xlsx
+++ b/data/papers_summary.xlsx
@@ -1,26 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kingsuca-my.sharepoint.com/personal/stephen_fan_kingsu_ca/Documents/01-Research/01-PaperProjects/InProgress/TokenizationSurvey/tokenization-survey/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephenfan/Library/CloudStorage/OneDrive-TheKing'sUniversity/01-Research/01-PaperProjects/InProgress/TokenizationSurvey/tokenization-survey/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="454" documentId="13_ncr:1_{9F290D21-0310-5947-9047-FFDB20A0199C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9C3EF01-15FF-7D49-AAE8-189F7FEA50CE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B5F13B3-EFAD-9D44-8A59-40BEC3922152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14080" yWindow="-21100" windowWidth="38400" windowHeight="21100" xr2:uid="{2EDFC2C0-EA07-B948-8B39-E25EA53281F4}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{2EDFC2C0-EA07-B948-8B39-E25EA53281F4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="ACM" sheetId="4" r:id="rId2"/>
-    <sheet name="ScienceDirect" sheetId="6" r:id="rId3"/>
-    <sheet name="Industrial" sheetId="3" r:id="rId4"/>
-    <sheet name="Stats" sheetId="2" r:id="rId5"/>
+    <sheet name="Summary" sheetId="7" r:id="rId1"/>
+    <sheet name="Summary-old" sheetId="1" r:id="rId2"/>
+    <sheet name="ACM" sheetId="4" r:id="rId3"/>
+    <sheet name="ScienceDirect" sheetId="6" r:id="rId4"/>
+    <sheet name="Industrial" sheetId="3" r:id="rId5"/>
+    <sheet name="Stats" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Summary!$K$1:$K$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Summary!$K$1:$K$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary-old'!$K$1:$K$114</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1752" uniqueCount="782">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2996" uniqueCount="910">
   <si>
     <t>Order</t>
   </si>
@@ -2537,6 +2539,392 @@
   </si>
   <si>
     <t>carbon emissions, Carbon-electricity, blockchain, deep learningalgorithms, heterogeneous data features</t>
+  </si>
+  <si>
+    <t>Token Smart contract details  designed but not implemented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZipZap is an
+ERC-1155 compliant solution which supports batch minting and transfer. It includes detailed of data to be tokenized. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bevin K.C., Ashu Verma
+</t>
+  </si>
+  <si>
+    <t>Hossein Saber, Tom Celig, Saber Talari, Wolfgang Ketter, Detlef Schoder</t>
+  </si>
+  <si>
+    <t>Blockchain, Hyperledger Fabric, AMM, Cryptocurrency</t>
+  </si>
+  <si>
+    <t>ERC-20/ERC-721</t>
+  </si>
+  <si>
+    <t>Blockchain, caliper, electric vehicle (EV), Ethereum, nonfungible tokens (NFTs), P2P energy trading</t>
+  </si>
+  <si>
+    <t>Peer-to-peer energy trading, Blockchain, Pricing scheme, Smart contract</t>
+  </si>
+  <si>
+    <t>Ajit Muzumdar, Chirag Modi, Madhu G.M.,  C. Vyjayanthi</t>
+  </si>
+  <si>
+    <t>Energy Internet, Blockchain, Energy Routing Protocols, Subscriber Matching, Energy-Efficient Path, Transmission Scheduling, Dynamic Routing, Peer-to-Peer Energy Trading, Distributed Energy Resources (DERs), Power Transmission Loss, Demand-Driven Energy System, Smart Contracts, Energy Tokenization, Decentralized Energy Systems, Secure Energy Exchange, Congestion Management</t>
+  </si>
+  <si>
+    <t>Binance Smart Chain</t>
+  </si>
+  <si>
+    <t>blockchain, tokenization, energy storage system, renewable energy, real-world asset, game theory, power purchase agreement</t>
+  </si>
+  <si>
+    <t>blockchain, energy attribute certificates, Energy Web Origin</t>
+  </si>
+  <si>
+    <t>PBFT  blockchain</t>
+  </si>
+  <si>
+    <t>ERC-721/ERC-1155</t>
+  </si>
+  <si>
+    <t>Self-sovereign Identity, Zero-Trust Security, Blockchain-enabled Transactive Energy, Green Energy, Energy Certificates, Concordium, IOTA Tangle</t>
+  </si>
+  <si>
+    <t>Blockchain, Sustainable energy certificates, IoT integration, Layer 2 scalability, Tokenized marketplace, Zero-knowledge proofs, AI analytics, Gamification, Energy transparency, Renewable energy trading</t>
+  </si>
+  <si>
+    <t>Renewable energy certificate, Blockchain, Privacy</t>
+  </si>
+  <si>
+    <t>Polygon Mumbai</t>
+  </si>
+  <si>
+    <t>ERC-20/ERC-721/ERC-4626</t>
+  </si>
+  <si>
+    <t>NFT/FT</t>
+  </si>
+  <si>
+    <t>Fabric Token SDK</t>
+  </si>
+  <si>
+    <t>ReFi Tokens</t>
+  </si>
+  <si>
+    <t>Yash Madhwal, Yury Yanovich, Matteo Coveri, Ninoslav Marina</t>
+  </si>
+  <si>
+    <t>Vaibhav Agarwal, Sujata Rani</t>
+  </si>
+  <si>
+    <t>Nan Ma, Alex Waegel, Max Hakkarainen, William W. Braham, Lior Glass, Dorit Aviv</t>
+  </si>
+  <si>
+    <t>M. Caruso, P. Gallo, M.G. Ippolito, S. Nassuato, N. Tomasone, E.R. Sanseverino, G. Sciumè, G. Zizzo</t>
+  </si>
+  <si>
+    <t>Manuel UtzSimon AlbrechtThorsten ZoernerJens Struker</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>Bulgaria, Romania, Greece, Belgium</t>
+  </si>
+  <si>
+    <t>Romania, Romania, Romania, Romania, Romania, Romania, Romania</t>
+  </si>
+  <si>
+    <t>India, India, India</t>
+  </si>
+  <si>
+    <t>Bangladesh, Bangladesh, Bangladesh</t>
+  </si>
+  <si>
+    <t>Canada, Canada, Canada</t>
+  </si>
+  <si>
+    <t>Turkey, Turkey, Turkey, Turkey</t>
+  </si>
+  <si>
+    <t>India, India</t>
+  </si>
+  <si>
+    <t>Germany, Germany, Germany, Germany, Germany</t>
+  </si>
+  <si>
+    <t>Germany, Germany, Germany, Germany</t>
+  </si>
+  <si>
+    <t>South Korea, South Korea, South Korea, South Korea</t>
+  </si>
+  <si>
+    <t>France, France</t>
+  </si>
+  <si>
+    <t>China, China, China</t>
+  </si>
+  <si>
+    <t>Australia, Australia, Australia</t>
+  </si>
+  <si>
+    <t>India, India, India, India, Canada, UAE</t>
+  </si>
+  <si>
+    <t>Canada, Canada</t>
+  </si>
+  <si>
+    <t>Singapore, Singapore, Singapore, Canada</t>
+  </si>
+  <si>
+    <t>India, India, India, India</t>
+  </si>
+  <si>
+    <t>Ireland, Ireland</t>
+  </si>
+  <si>
+    <t>Spain, UK, UK, Spain,, Spain</t>
+  </si>
+  <si>
+    <t>Iran, Iran</t>
+  </si>
+  <si>
+    <t>Thailand, Thailand</t>
+  </si>
+  <si>
+    <t>Australia, Australia, Australia, Norway, Australia, Australia, Australia, Qatar</t>
+  </si>
+  <si>
+    <t>India, India, India, India, India, India</t>
+  </si>
+  <si>
+    <t>Sri Lanka, Sri Lanka, Sri Lanka, Sri Lanka, Sri Lanka, Sri Lanka, New Zealand</t>
+  </si>
+  <si>
+    <t>Romania, Romania, Romania,Romania</t>
+  </si>
+  <si>
+    <t>Russia, Russia, Switzerland</t>
+  </si>
+  <si>
+    <t>Turkey, Turkey</t>
+  </si>
+  <si>
+    <t>Ireland, Ireland, Ireland</t>
+  </si>
+  <si>
+    <t>India, USA, India, India, India</t>
+  </si>
+  <si>
+    <t>China, China, China, China, China, China</t>
+  </si>
+  <si>
+    <t>Bulgaria, Bulgaria</t>
+  </si>
+  <si>
+    <t>China, China</t>
+  </si>
+  <si>
+    <t>Singapore, Singapore, Singapore, Singapore, Singapore</t>
+  </si>
+  <si>
+    <t>Brazil, Brazil, Brazil</t>
+  </si>
+  <si>
+    <t>Taiwan, Taiwan, UK</t>
+  </si>
+  <si>
+    <t>Germany, Germany, Germany</t>
+  </si>
+  <si>
+    <t>Indonesia, Indonesia, Indonesia, Indonesia, Indonesia, Indonesia, Indonesia, Indonesia, Indonesia, Netherlands</t>
+  </si>
+  <si>
+    <t>China, China, China, China, China</t>
+  </si>
+  <si>
+    <t>Norway, USA,  USA, Turkey, Tailand,  USA</t>
+  </si>
+  <si>
+    <t>India, India, Saudi Arabia, Saudi Arabia, India, India</t>
+  </si>
+  <si>
+    <t>Brazil, Brazil, Brazil, Brazil, Brazil, Brazil</t>
+  </si>
+  <si>
+    <t>Bangladesh, Bangladesh, Bangladesh, Bangladesh</t>
+  </si>
+  <si>
+    <t>Denmark, Denmark, Pakistan, Pakistan</t>
+  </si>
+  <si>
+    <t>Australia, Australia, Australia, Singapore, Singapore</t>
+  </si>
+  <si>
+    <t>UK, UK, UK, Singapore, Singapore</t>
+  </si>
+  <si>
+    <t>Spain, Spain</t>
+  </si>
+  <si>
+    <t>Australia, Australia, Australia, Australia</t>
+  </si>
+  <si>
+    <t>India, India, India, India, India, Iraq</t>
+  </si>
+  <si>
+    <t>Romania, Romania, Romania</t>
+  </si>
+  <si>
+    <t>Romania, Romania, Romania,Romania, Romania,  Romania, Romania, Italy, Italy, Italy, Italy, Italy, Italy</t>
+  </si>
+  <si>
+    <t>Denmark, Denmark, Denmark, Denmark, China</t>
+  </si>
+  <si>
+    <t>Denmark, Denmark</t>
+  </si>
+  <si>
+    <t>Norway,Norway, Norway</t>
+  </si>
+  <si>
+    <t>China, China, China, China, Canada, USA</t>
+  </si>
+  <si>
+    <t>Italy, Italy</t>
+  </si>
+  <si>
+    <t>Australia, Australia</t>
+  </si>
+  <si>
+    <t>India, India, India, India, Uzbekistan</t>
+  </si>
+  <si>
+    <t>Haseeb Saeed, Syed Muhammad Danish, Kaiwen Zhang</t>
+  </si>
+  <si>
+    <t>R Udayakumar, A Haja Alaudeen, Anjali Goswami, N Arvinth, G Abdumalikova</t>
+  </si>
+  <si>
+    <t>Nan Wang, Sid Chi-Kin Chau</t>
+  </si>
+  <si>
+    <t>Singapore, China, China</t>
+  </si>
+  <si>
+    <t>Yunshu Liu, Man Hon Cheung, Jianwei Huang</t>
+  </si>
+  <si>
+    <t>Chunliang Lin</t>
+  </si>
+  <si>
+    <t>Lianghaojie Zhou, Yipeng Yang, Xin Li, Youquan Xian, Dongcheng Li, Peng Liu</t>
+  </si>
+  <si>
+    <t>Ye Chen, Peilin Wu, Yuanliang Li, Peng Zhang, Jun Yan, Mohsen Ghafouri, Yuhong Liu</t>
+  </si>
+  <si>
+    <t>USA, China, Canada, China, Canada, Canada, USA</t>
+  </si>
+  <si>
+    <t>Chunzhe Li, Lingjiang Zhai, Keqiang Wang, Zhansheng Zhang, Chengkang Zhang, Xue Li</t>
+  </si>
+  <si>
+    <t>Emanuele Antonio Napoli, Valentina Gatteschi</t>
+  </si>
+  <si>
+    <t>Michell Boerger, Philipp Lämmel, Nikolay Tcholtchev, Manfred Hauswirth</t>
+  </si>
+  <si>
+    <t>Jivtesh M R, Rohit Mathew Samuel, Gaushik M R, Siddhi Menon, Sai Shibu N B, Sethuraman N Rao</t>
+  </si>
+  <si>
+    <t>Rong Chen</t>
+  </si>
+  <si>
+    <t>Nan Wang, Sid Chi-Kin Chau, Yue Zhou</t>
+  </si>
+  <si>
+    <t>Vinod Pangracious</t>
+  </si>
+  <si>
+    <t>UAE</t>
+  </si>
+  <si>
+    <t>Sid Chi-Kin Chau, Yue Zhou</t>
+  </si>
+  <si>
+    <t>Johannes Sedlmeir, Fabiane Völter, Jens Struker</t>
+  </si>
+  <si>
+    <t>Shengnan Zhang, Jiaxing Xuan, Zitong Lyu, Yuchen Fu</t>
+  </si>
+  <si>
+    <t>China, China, China, China</t>
+  </si>
+  <si>
+    <t>Riseul Ryu, Soonja Yeom</t>
+  </si>
+  <si>
+    <t>Spain, Spain, Spain, Spain, Spain, Spain, Spain, Spain</t>
+  </si>
+  <si>
+    <t>Vietnam, Vietnam, Vietnam</t>
+  </si>
+  <si>
+    <t>Vietnam, Vietnam, Vietnam, Vietnam, Vietnam, Vietnam, Vietnam, Vietnam</t>
+  </si>
+  <si>
+    <t>Spain, Spain, Spain, Spain</t>
+  </si>
+  <si>
+    <t>Germany, Germany</t>
+  </si>
+  <si>
+    <t>Russia</t>
+  </si>
+  <si>
+    <t>Iran, Iran,  Iran</t>
+  </si>
+  <si>
+    <t>USA, USA, USA, USA,China</t>
+  </si>
+  <si>
+    <t>Iran, Iran, Denmark</t>
+  </si>
+  <si>
+    <t>Russia, Russia, Switzerland, Macedonia</t>
+  </si>
+  <si>
+    <t>India, India, India, Iran, Jordan</t>
+  </si>
+  <si>
+    <t>China, China, China, Ghana, Ghana</t>
+  </si>
+  <si>
+    <t>Saudi Arabia</t>
+  </si>
+  <si>
+    <t>USA, USA, USA, USA,USA, USA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">China, China, China, China, France, New Zealand, Australia </t>
+  </si>
+  <si>
+    <t>India, India, USA</t>
+  </si>
+  <si>
+    <t>Australia, Ghana</t>
+  </si>
+  <si>
+    <t>Italy, Italy, Italy, Italy, Italy, Italy, Italy, Italy</t>
   </si>
 </sst>
 </file>
@@ -3048,6 +3436,4321 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FE52559-3A19-114C-BEE9-43E5B99405E2}">
+  <dimension ref="A1:L113"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="3" max="3" width="26.33203125" customWidth="1"/>
+    <col min="4" max="4" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38" customWidth="1"/>
+    <col min="6" max="6" width="134" customWidth="1"/>
+    <col min="12" max="12" width="28" style="6" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="136" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>782</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="170" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2019</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>775</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="221" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>783</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="187" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>778</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="170" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>784</v>
+      </c>
+      <c r="D7" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="204" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>785</v>
+      </c>
+      <c r="D8" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="136" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="204" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>786</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="187" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="204" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="170" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>787</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D14" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>788</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="136" x14ac:dyDescent="0.2">
+      <c r="A15" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>789</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="170" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>776</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A18" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>790</v>
+      </c>
+      <c r="D18" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="204" x14ac:dyDescent="0.2">
+      <c r="A19" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D19" s="6">
+        <v>2019</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="289" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" s="6">
+        <v>2019</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="D21" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="170" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="D22" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>791</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="204" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="D23" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="D24" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="204" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="D25" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="153" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="D26" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="289" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="D27" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="388" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="D28" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="153" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="D29" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>792</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="D30" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L30" s="6" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A31" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="D31" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="136" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="D32" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A33" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="D33" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>793</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="170" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="D34" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="238" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="D35" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="221" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="D36" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A37" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="D37" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D38" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D39" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="153" x14ac:dyDescent="0.2">
+      <c r="A40" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D40" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J40" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="187" x14ac:dyDescent="0.2">
+      <c r="A41" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D41" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L41" s="6" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="289" x14ac:dyDescent="0.2">
+      <c r="A42" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="D42" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I42" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J42" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L42" s="6" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A43" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D43" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>794</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L43" s="6" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D44" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L44" s="6" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="340" x14ac:dyDescent="0.2">
+      <c r="A45" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D45" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="K45" s="6" t="s">
+        <v>776</v>
+      </c>
+      <c r="L45" s="6" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A46" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D46" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I46" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J46" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="K46" s="6" t="s">
+        <v>778</v>
+      </c>
+      <c r="L46" s="6" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A47" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D47" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>795</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="L47" s="6" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A48" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D48" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I48" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J48" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="K48" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L48" s="6" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" ht="372" x14ac:dyDescent="0.2">
+      <c r="A49" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D49" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I49" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J49" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="K49" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L49" s="6" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A50" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D50" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="G50" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I50" s="6" t="s">
+        <v>796</v>
+      </c>
+      <c r="J50" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="K50" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L50" s="6" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" ht="170" x14ac:dyDescent="0.2">
+      <c r="A51" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D51" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I51" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J51" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="K51" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L51" s="6" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A52" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D52" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J52" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="K52" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L52" s="6" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A53" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="D53" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>797</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="G53" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I53" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J53" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="L53" s="6" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" ht="221" x14ac:dyDescent="0.2">
+      <c r="A54" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D54" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>798</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I54" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J54" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="K54" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="L54" s="6" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A55" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="D55" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J55" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="K55" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L55" s="6" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+      <c r="A56" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="D56" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>799</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="G56" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="I56" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J56" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K56" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="L56" s="6" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A57" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D57" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="G57" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H57" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I57" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J57" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="K57" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L57" s="6" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" ht="372" x14ac:dyDescent="0.2">
+      <c r="A58" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="D58" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I58" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J58" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="K58" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L58" s="6" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A59" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="D59" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>800</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I59" s="6" t="s">
+        <v>801</v>
+      </c>
+      <c r="J59" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="K59" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L59" s="6" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" ht="187" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="D60" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="G60" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I60" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J60" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="K60" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L60" s="6" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" ht="404" x14ac:dyDescent="0.2">
+      <c r="A61" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D61" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="G61" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H61" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I61" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J61" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="K61" s="6" t="s">
+        <v>776</v>
+      </c>
+      <c r="L61" s="6" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A62" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="D62" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E62" s="6" t="s">
+        <v>728</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="G62" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H62" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I62" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J62" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="K62" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L62" s="6" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" ht="204" x14ac:dyDescent="0.2">
+      <c r="A63" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D63" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="F63" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="G63" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H63" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I63" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J63" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="K63" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L63" s="6" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" ht="238" x14ac:dyDescent="0.2">
+      <c r="A64" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="D64" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="G64" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H64" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I64" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J64" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="K64" s="6" t="s">
+        <v>776</v>
+      </c>
+      <c r="L64" s="6" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+      <c r="A65" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="D65" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="G65" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H65" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I65" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J65" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="K65" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L65" s="6" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" ht="170" x14ac:dyDescent="0.2">
+      <c r="A66" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="D66" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="G66" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I66" s="6" t="s">
+        <v>802</v>
+      </c>
+      <c r="J66" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="K66" s="6" t="s">
+        <v>776</v>
+      </c>
+      <c r="L66" s="6" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" ht="238" x14ac:dyDescent="0.2">
+      <c r="A67" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="D67" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="G67" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H67" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I67" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J67" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="K67" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L67" s="6" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A68" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="D68" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>478</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="G68" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I68" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J68" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="K68" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L68" s="6" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A69" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>872</v>
+      </c>
+      <c r="D69" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="G69" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I69" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J69" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="K69" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L69" s="6" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" ht="289" x14ac:dyDescent="0.2">
+      <c r="A70" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>871</v>
+      </c>
+      <c r="D70" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I70" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J70" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="K70" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L70" s="6" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" ht="238" x14ac:dyDescent="0.2">
+      <c r="A71" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>870</v>
+      </c>
+      <c r="D71" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="G71" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="H71" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I71" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="J71" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="K71" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L71" s="6" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A72" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>874</v>
+      </c>
+      <c r="D72" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="G72" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I72" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J72" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="K72" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L72" s="6" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A73" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>875</v>
+      </c>
+      <c r="D73" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="G73" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H73" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I73" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J73" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="K73" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L73" s="6" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A74" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>876</v>
+      </c>
+      <c r="D74" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="G74" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I74" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J74" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="K74" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L74" s="6" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" ht="238" x14ac:dyDescent="0.2">
+      <c r="A75" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>877</v>
+      </c>
+      <c r="D75" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="G75" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H75" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I75" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J75" s="6" t="s">
+        <v>431</v>
+      </c>
+      <c r="K75" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L75" s="6" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A76" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>879</v>
+      </c>
+      <c r="D76" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>781</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="G76" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H76" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I76" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J76" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="K76" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L76" s="6" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A77" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>880</v>
+      </c>
+      <c r="D77" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>513</v>
+      </c>
+      <c r="G77" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H77" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I77" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J77" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="K77" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L77" s="6" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" ht="238" x14ac:dyDescent="0.2">
+      <c r="A78" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>881</v>
+      </c>
+      <c r="D78" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="G78" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H78" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I78" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J78" s="6" t="s">
+        <v>440</v>
+      </c>
+      <c r="K78" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L78" s="6" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A79" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>882</v>
+      </c>
+      <c r="D79" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="G79" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I79" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J79" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="K79" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L79" s="6" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" ht="221" x14ac:dyDescent="0.2">
+      <c r="A80" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>883</v>
+      </c>
+      <c r="D80" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="G80" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H80" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I80" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J80" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="K80" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L80" s="6" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A81" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>884</v>
+      </c>
+      <c r="D81" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E81" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="G81" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H81" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J81" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="K81" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L81" s="6" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" ht="289" x14ac:dyDescent="0.2">
+      <c r="A82" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>887</v>
+      </c>
+      <c r="D82" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="G82" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H82" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I82" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J82" s="6" t="s">
+        <v>452</v>
+      </c>
+      <c r="K82" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L82" s="6" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A83" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>885</v>
+      </c>
+      <c r="D83" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E83" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="F83" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="G83" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H83" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I83" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J83" s="6" t="s">
+        <v>455</v>
+      </c>
+      <c r="K83" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L83" s="6" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A84" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>884</v>
+      </c>
+      <c r="D84" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E84" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="F84" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="G84" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I84" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J84" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="K84" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L84" s="6" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A85" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>888</v>
+      </c>
+      <c r="D85" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E85" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="F85" s="6" t="s">
+        <v>521</v>
+      </c>
+      <c r="G85" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H85" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I85" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J85" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="K85" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L85" s="6" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" ht="306" x14ac:dyDescent="0.2">
+      <c r="A86" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>889</v>
+      </c>
+      <c r="D86" s="6">
+        <v>2020</v>
+      </c>
+      <c r="E86" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="F86" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="G86" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H86" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I86" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J86" s="6" t="s">
+        <v>464</v>
+      </c>
+      <c r="K86" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L86" s="6" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A87" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>891</v>
+      </c>
+      <c r="D87" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E87" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="G87" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H87" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I87" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J87" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="K87" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L87" s="6" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" ht="306" x14ac:dyDescent="0.2">
+      <c r="A88" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="D88" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F88" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G88" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H88" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I88" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J88" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="K88" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="L88" s="6" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A89" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>537</v>
+      </c>
+      <c r="D89" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="F89" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H89" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I89" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J89" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="K89" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="L89" s="6" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A90" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="D90" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E90" s="6" t="s">
+        <v>547</v>
+      </c>
+      <c r="F90" s="6" t="s">
+        <v>546</v>
+      </c>
+      <c r="G90" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H90" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I90" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J90" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="K90" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="L90" s="6" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A91" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>550</v>
+      </c>
+      <c r="D91" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>551</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>549</v>
+      </c>
+      <c r="G91" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="H91" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I91" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J91" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="K91" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="L91" s="6" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A92" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="D92" s="6">
+        <v>2020</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="F92" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="G92" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H92" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I92" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J92" s="6" t="s">
+        <v>553</v>
+      </c>
+      <c r="K92" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="L92" s="6" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A93" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>809</v>
+      </c>
+      <c r="D93" s="6">
+        <v>2019</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>557</v>
+      </c>
+      <c r="F93" s="6" t="s">
+        <v>556</v>
+      </c>
+      <c r="G93" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H93" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I93" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J93" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="K93" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="L93" s="6" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" ht="372" x14ac:dyDescent="0.2">
+      <c r="A94" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>683</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>565</v>
+      </c>
+      <c r="D94" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>713</v>
+      </c>
+      <c r="F94" s="6" t="s">
+        <v>714</v>
+      </c>
+      <c r="G94" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="H94" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I94" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J94" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="K94" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L94" s="6" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" ht="372" x14ac:dyDescent="0.2">
+      <c r="A95" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>684</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>573</v>
+      </c>
+      <c r="D95" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E95" s="6" t="s">
+        <v>717</v>
+      </c>
+      <c r="F95" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="G95" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H95" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I95" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J95" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="K95" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L95" s="6" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" ht="323" x14ac:dyDescent="0.2">
+      <c r="A96" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>580</v>
+      </c>
+      <c r="D96" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E96" s="6" t="s">
+        <v>720</v>
+      </c>
+      <c r="F96" s="6" t="s">
+        <v>721</v>
+      </c>
+      <c r="G96" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="H96" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I96" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J96" s="6" t="s">
+        <v>583</v>
+      </c>
+      <c r="K96" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L96" s="6" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" ht="323" x14ac:dyDescent="0.2">
+      <c r="A97" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="D97" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E97" s="6" t="s">
+        <v>722</v>
+      </c>
+      <c r="F97" s="6" t="s">
+        <v>723</v>
+      </c>
+      <c r="G97" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H97" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I97" s="6" t="s">
+        <v>803</v>
+      </c>
+      <c r="J97" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="K97" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L97" s="6" t="s">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" ht="289" x14ac:dyDescent="0.2">
+      <c r="A98" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>687</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="D98" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E98" s="6" t="s">
+        <v>724</v>
+      </c>
+      <c r="F98" s="6" t="s">
+        <v>725</v>
+      </c>
+      <c r="G98" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H98" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I98" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J98" s="6" t="s">
+        <v>591</v>
+      </c>
+      <c r="K98" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L98" s="6" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" ht="356" x14ac:dyDescent="0.2">
+      <c r="A99" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="D99" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>726</v>
+      </c>
+      <c r="F99" s="6" t="s">
+        <v>727</v>
+      </c>
+      <c r="G99" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H99" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I99" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J99" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="K99" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L99" s="6" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12" ht="221" x14ac:dyDescent="0.2">
+      <c r="A100" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="D100" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E100" s="6" t="s">
+        <v>730</v>
+      </c>
+      <c r="F100" s="6" t="s">
+        <v>731</v>
+      </c>
+      <c r="G100" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H100" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I100" s="6" t="s">
+        <v>804</v>
+      </c>
+      <c r="J100" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="K100" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L100" s="6" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" ht="323" x14ac:dyDescent="0.2">
+      <c r="A101" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>805</v>
+      </c>
+      <c r="D101" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E101" s="6" t="s">
+        <v>732</v>
+      </c>
+      <c r="F101" s="6" t="s">
+        <v>733</v>
+      </c>
+      <c r="G101" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H101" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I101" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J101" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="K101" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L101" s="6" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" ht="289" x14ac:dyDescent="0.2">
+      <c r="A102" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>692</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>611</v>
+      </c>
+      <c r="D102" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E102" s="6" t="s">
+        <v>736</v>
+      </c>
+      <c r="F102" s="6" t="s">
+        <v>737</v>
+      </c>
+      <c r="G102" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H102" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I102" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J102" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="K102" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L102" s="6" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A103" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>806</v>
+      </c>
+      <c r="D103" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>738</v>
+      </c>
+      <c r="F103" s="6" t="s">
+        <v>739</v>
+      </c>
+      <c r="G103" s="6" t="s">
+        <v>615</v>
+      </c>
+      <c r="H103" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I103" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J103" s="6" t="s">
+        <v>617</v>
+      </c>
+      <c r="K103" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L103" s="6" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" ht="388" x14ac:dyDescent="0.2">
+      <c r="A104" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>695</v>
+      </c>
+      <c r="C104" s="6" t="s">
+        <v>621</v>
+      </c>
+      <c r="D104" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E104" s="6" t="s">
+        <v>742</v>
+      </c>
+      <c r="F104" s="6" t="s">
+        <v>743</v>
+      </c>
+      <c r="G104" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H104" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I104" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J104" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="K104" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L104" s="6" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A105" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>696</v>
+      </c>
+      <c r="C105" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="D105" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E105" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="F105" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="G105" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H105" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="I105" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J105" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="K105" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L105" s="6" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" ht="388" x14ac:dyDescent="0.2">
+      <c r="A106" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>697</v>
+      </c>
+      <c r="C106" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="D106" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E106" s="6" t="s">
+        <v>746</v>
+      </c>
+      <c r="F106" s="6" t="s">
+        <v>747</v>
+      </c>
+      <c r="G106" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H106" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I106" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J106" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="K106" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L106" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12" ht="388" x14ac:dyDescent="0.2">
+      <c r="A107" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B107" s="6" t="s">
+        <v>698</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="D107" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E107" s="6" t="s">
+        <v>748</v>
+      </c>
+      <c r="F107" s="6" t="s">
+        <v>749</v>
+      </c>
+      <c r="G107" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H107" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I107" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J107" s="6" t="s">
+        <v>637</v>
+      </c>
+      <c r="K107" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L107" s="6" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" ht="404" x14ac:dyDescent="0.2">
+      <c r="A108" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B108" s="6" t="s">
+        <v>700</v>
+      </c>
+      <c r="C108" s="6" t="s">
+        <v>807</v>
+      </c>
+      <c r="D108" s="6">
+        <v>2023</v>
+      </c>
+      <c r="E108" s="6" t="s">
+        <v>752</v>
+      </c>
+      <c r="F108" s="6" t="s">
+        <v>753</v>
+      </c>
+      <c r="G108" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H108" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I108" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J108" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="K108" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L108" s="6" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" ht="340" x14ac:dyDescent="0.2">
+      <c r="A109" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B109" s="6" t="s">
+        <v>702</v>
+      </c>
+      <c r="C109" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="D109" s="6">
+        <v>2026</v>
+      </c>
+      <c r="E109" s="6" t="s">
+        <v>756</v>
+      </c>
+      <c r="F109" s="6" t="s">
+        <v>757</v>
+      </c>
+      <c r="G109" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H109" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I109" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J109" s="6" t="s">
+        <v>651</v>
+      </c>
+      <c r="K109" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L109" s="6" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" ht="356" x14ac:dyDescent="0.2">
+      <c r="A110" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B110" s="6" t="s">
+        <v>704</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="D110" s="6">
+        <v>2022</v>
+      </c>
+      <c r="E110" s="6" t="s">
+        <v>760</v>
+      </c>
+      <c r="F110" s="6" t="s">
+        <v>761</v>
+      </c>
+      <c r="G110" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H110" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I110" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J110" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="K110" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L110" s="6" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12" ht="340" x14ac:dyDescent="0.2">
+      <c r="A111" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B111" s="6" t="s">
+        <v>706</v>
+      </c>
+      <c r="C111" s="6" t="s">
+        <v>662</v>
+      </c>
+      <c r="D111" s="6">
+        <v>2024</v>
+      </c>
+      <c r="E111" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="F111" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="G111" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H111" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I111" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J111" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="K111" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L111" s="6" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" ht="323" x14ac:dyDescent="0.2">
+      <c r="A112" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B112" s="6" t="s">
+        <v>708</v>
+      </c>
+      <c r="C112" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="D112" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E112" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="F112" s="6" t="s">
+        <v>769</v>
+      </c>
+      <c r="G112" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H112" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="I112" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J112" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="K112" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L112" s="6" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12" ht="340" x14ac:dyDescent="0.2">
+      <c r="A113" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B113" s="6" t="s">
+        <v>709</v>
+      </c>
+      <c r="C113" s="6" t="s">
+        <v>808</v>
+      </c>
+      <c r="D113" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E113" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="F113" s="6" t="s">
+        <v>772</v>
+      </c>
+      <c r="G113" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H113" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="I113" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J113" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="K113" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L113" s="6" t="s">
+        <v>909</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="K1:K113" xr:uid="{4FE52559-3A19-114C-BEE9-43E5B99405E2}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BAEB69D-E09B-E34E-B100-9FBAB6BE6E2D}">
   <dimension ref="A1:Z114"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -7094,7 +11797,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D7C1615-AFD7-1B43-AE24-5719B5805A5F}">
   <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="274" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -8015,7 +12718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4A1DF10-A716-BD49-BE5F-DFE8365D4EFD}">
   <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="25.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -9121,7 +13824,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C8611A3-78B5-7A45-8D81-8170174AEEE1}">
   <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -9307,7 +14010,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36B7C806-E0E8-8B49-8105-BDB87BE43735}">
   <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>